<commit_message>
Base.xlsx：arg1・arg2 を refersTo の下位属性 retrieve の下位属性にする（追記R774）。argument・taskArg1・taskArg2 を外す
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ontology/Base.xlsx
+++ b/ontology/Base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\home\doc\PLR\dist\schemata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6EE464-1EAC-42B5-B1DF-B18A6CF4523E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA3F03A-7DCA-4B8A-9F7C-161952D9B303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="15576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="124">
   <si>
     <t>dateTime</t>
   </si>
@@ -374,10 +374,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>argument ja:項;argument</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>index(1 ja:検索キー;retrieval key|||[]</t>
     <phoneticPr fontId="2"/>
   </si>
@@ -397,27 +393,11 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>argument1 ja:第1項;argument1</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>argument2 ja:第2項;argument2</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>arg1</t>
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>taskArg1</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>arg2</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>taskArg2</t>
     <phoneticPr fontId="2"/>
   </si>
   <si>
@@ -482,6 +462,14 @@
   </si>
   <si>
     <t>Channel</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>refersTo</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>retrieve retrieve</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -537,13 +525,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF00B0F0"/>
-      <name val="Meiryo UI"/>
-      <family val="3"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="メイリオ"/>
       <family val="3"/>
       <charset val="128"/>
@@ -579,6 +560,12 @@
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Meiryo"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Meiryo UI"/>
       <family val="3"/>
       <charset val="128"/>
     </font>
@@ -859,7 +846,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -958,19 +945,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -979,75 +960,57 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1069,7 +1032,31 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1081,8 +1068,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCCFFFF"/>
       <color rgb="FFFFFFCC"/>
-      <color rgb="FFCCFFFF"/>
     </mruColors>
   </colors>
   <extLst>
@@ -1393,7 +1380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30509B9C-F985-4EE4-8893-AAEEF9CB070C}">
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="16.2"/>
   <cols>
     <col min="1" max="1" width="38.88671875" style="17" customWidth="1"/>
@@ -1405,21 +1392,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.6" customHeight="1">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="52" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="44"/>
+      <c r="B1" s="53"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="57" t="s">
-        <v>125</v>
-      </c>
-      <c r="E1" s="57"/>
-      <c r="F1" s="57"/>
-      <c r="G1" s="57"/>
-      <c r="H1" s="57"/>
+      <c r="D1" s="47" t="s">
+        <v>120</v>
+      </c>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
     </row>
     <row r="2" spans="1:8" ht="39" customHeight="1">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="54" t="s">
         <v>86</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1428,14 +1415,14 @@
       <c r="C2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="63"/>
+      <c r="A3" s="55"/>
       <c r="B3" s="5" t="s">
         <v>90</v>
       </c>
@@ -1445,7 +1432,7 @@
       <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="63"/>
+      <c r="A4" s="55"/>
       <c r="B4" s="21" t="s">
         <v>1</v>
       </c>
@@ -1455,7 +1442,7 @@
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="63"/>
+      <c r="A5" s="55"/>
       <c r="B5" s="23" t="s">
         <v>73</v>
       </c>
@@ -1465,8 +1452,8 @@
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="63"/>
-      <c r="B6" s="64" t="s">
+      <c r="A6" s="55"/>
+      <c r="B6" s="56" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1475,23 +1462,23 @@
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="63"/>
-      <c r="B7" s="65"/>
+      <c r="A7" s="55"/>
+      <c r="B7" s="57"/>
       <c r="C7" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="63"/>
-      <c r="B8" s="66"/>
+      <c r="A8" s="55"/>
+      <c r="B8" s="58"/>
       <c r="C8" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="63"/>
+      <c r="A9" s="55"/>
       <c r="B9" s="7" t="s">
         <v>7</v>
       </c>
@@ -1501,8 +1488,8 @@
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="63"/>
-      <c r="B10" s="67" t="s">
+      <c r="A10" s="55"/>
+      <c r="B10" s="59" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -1511,15 +1498,15 @@
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="63"/>
-      <c r="B11" s="68"/>
+      <c r="A11" s="55"/>
+      <c r="B11" s="60"/>
       <c r="C11" s="7" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="63"/>
+      <c r="A12" s="55"/>
       <c r="B12" s="18" t="s">
         <v>57</v>
       </c>
@@ -1529,48 +1516,48 @@
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="16.2" customHeight="1">
-      <c r="A13" s="63"/>
-      <c r="B13" s="69" t="s">
-        <v>103</v>
-      </c>
-      <c r="C13" s="39" t="s">
-        <v>111</v>
+      <c r="A13" s="55"/>
+      <c r="B13" s="61" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="16.2" customHeight="1">
-      <c r="A14" s="35"/>
-      <c r="B14" s="69"/>
-      <c r="C14" s="40" t="s">
-        <v>102</v>
+      <c r="A14" s="33"/>
+      <c r="B14" s="61"/>
+      <c r="C14" s="38" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="35"/>
-      <c r="B15" s="69"/>
-      <c r="C15" s="58" t="s">
-        <v>120</v>
-      </c>
-      <c r="D15" s="41" t="s">
-        <v>121</v>
-      </c>
-      <c r="E15" s="60" t="s">
-        <v>123</v>
+      <c r="A15" s="33"/>
+      <c r="B15" s="61"/>
+      <c r="C15" s="48" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="39" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="50" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="35"/>
-      <c r="B16" s="69"/>
-      <c r="C16" s="59"/>
-      <c r="D16" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="E16" s="60"/>
+      <c r="A16" s="33"/>
+      <c r="B16" s="61"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="40" t="s">
+        <v>117</v>
+      </c>
+      <c r="E16" s="50"/>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="37" t="s">
+      <c r="B17" s="35" t="s">
         <v>92</v>
       </c>
       <c r="C17" s="2"/>
@@ -1581,26 +1568,26 @@
         <v>95</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="53" t="s">
+      <c r="A19" s="41" t="s">
         <v>62</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="64.8">
-      <c r="A20" s="53"/>
+      <c r="A20" s="41"/>
       <c r="B20" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>64</v>
@@ -1608,7 +1595,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="8" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B21" s="29" t="s">
         <v>94</v>
@@ -1661,519 +1648,495 @@
       <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4" ht="17.399999999999999">
-      <c r="A27" s="54" t="s">
+      <c r="A27" s="42" t="s">
+        <v>107</v>
+      </c>
+      <c r="B27" s="36" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+    </row>
+    <row r="28" spans="1:4" ht="17.399999999999999">
+      <c r="A28" s="43"/>
+      <c r="B28" s="36" t="s">
+        <v>109</v>
+      </c>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+    </row>
+    <row r="29" spans="1:4" ht="17.399999999999999">
+      <c r="A29" s="43"/>
+      <c r="B29" s="36" t="s">
+        <v>119</v>
+      </c>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+    </row>
+    <row r="30" spans="1:4" ht="17.399999999999999">
+      <c r="A30" s="43"/>
+      <c r="B30" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+    </row>
+    <row r="31" spans="1:4" ht="17.399999999999999">
+      <c r="A31" s="43"/>
+      <c r="B31" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+    </row>
+    <row r="32" spans="1:4" ht="17.399999999999999">
+      <c r="A32" s="43"/>
+      <c r="B32" s="36" t="s">
         <v>112</v>
       </c>
-      <c r="B27" s="38" t="s">
-        <v>119</v>
-      </c>
-      <c r="C27" s="34"/>
-      <c r="D27" s="34"/>
-    </row>
-    <row r="28" spans="1:4" ht="17.399999999999999">
-      <c r="A28" s="55"/>
-      <c r="B28" s="38" t="s">
-        <v>114</v>
-      </c>
-      <c r="C28" s="34"/>
-      <c r="D28" s="34"/>
-    </row>
-    <row r="29" spans="1:4" ht="17.399999999999999">
-      <c r="A29" s="55"/>
-      <c r="B29" s="38" t="s">
-        <v>124</v>
-      </c>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-    </row>
-    <row r="30" spans="1:4" ht="17.399999999999999">
-      <c r="A30" s="55"/>
-      <c r="B30" s="38" t="s">
-        <v>115</v>
-      </c>
-      <c r="C30" s="34"/>
-      <c r="D30" s="34"/>
-    </row>
-    <row r="31" spans="1:4" ht="17.399999999999999">
-      <c r="A31" s="55"/>
-      <c r="B31" s="38" t="s">
-        <v>116</v>
-      </c>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-    </row>
-    <row r="32" spans="1:4" ht="17.399999999999999">
-      <c r="A32" s="55"/>
-      <c r="B32" s="38" t="s">
-        <v>117</v>
-      </c>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
     </row>
     <row r="33" spans="1:4" ht="17.399999999999999">
-      <c r="A33" s="55"/>
-      <c r="B33" s="38" t="s">
-        <v>118</v>
-      </c>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
+      <c r="A33" s="43"/>
+      <c r="B33" s="36" t="s">
+        <v>113</v>
+      </c>
+      <c r="C33" s="32"/>
+      <c r="D33" s="32"/>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="33" t="s">
-        <v>99</v>
-      </c>
-      <c r="B34" s="32"/>
-      <c r="C34" s="2"/>
+      <c r="A34" s="63" t="s">
+        <v>122</v>
+      </c>
+      <c r="B34" s="68" t="s">
+        <v>123</v>
+      </c>
+      <c r="C34" s="34" t="s">
+        <v>104</v>
+      </c>
       <c r="D34" s="2"/>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="45" t="s">
+      <c r="A35" s="67"/>
+      <c r="B35" s="69"/>
+      <c r="C35" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="36" t="s">
-        <v>107</v>
-      </c>
-      <c r="C35" s="2"/>
       <c r="D35" s="2"/>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" s="46"/>
-      <c r="B36" s="36" t="s">
-        <v>108</v>
+      <c r="A36" s="64" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" s="26" t="s">
+        <v>64</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="45" t="s">
-        <v>106</v>
-      </c>
-      <c r="B37" s="36" t="s">
-        <v>109</v>
-      </c>
-      <c r="C37" s="2"/>
+      <c r="A37" s="65"/>
+      <c r="B37" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>79</v>
+      </c>
       <c r="D37" s="2"/>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="46"/>
-      <c r="B38" s="36" t="s">
-        <v>110</v>
-      </c>
-      <c r="C38" s="2"/>
+      <c r="A38" s="65"/>
+      <c r="B38" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>85</v>
+      </c>
       <c r="D38" s="2"/>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="47" t="s">
-        <v>77</v>
-      </c>
-      <c r="B39" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="C39" s="2"/>
+      <c r="A39" s="65"/>
+      <c r="B39" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>81</v>
+      </c>
       <c r="D39" s="2"/>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="48"/>
+      <c r="A40" s="66"/>
       <c r="B40" s="25" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D40" s="2"/>
     </row>
     <row r="41" spans="1:4">
-      <c r="A41" s="48"/>
-      <c r="B41" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>85</v>
-      </c>
+      <c r="A41" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="C41" s="2"/>
       <c r="D41" s="2"/>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="48"/>
+      <c r="A42" s="28" t="s">
+        <v>75</v>
+      </c>
       <c r="B42" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>81</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="C42" s="2"/>
       <c r="D42" s="2"/>
     </row>
     <row r="43" spans="1:4">
-      <c r="A43" s="49"/>
-      <c r="B43" s="25" t="s">
-        <v>82</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>83</v>
-      </c>
+      <c r="A43" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C43" s="2"/>
       <c r="D43" s="2"/>
     </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="24" t="s">
-        <v>63</v>
+    <row r="44" spans="1:4" ht="32.4">
+      <c r="A44" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>53</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="B45" s="25" t="s">
-        <v>76</v>
-      </c>
+      <c r="A45" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:4">
+    <row r="46" spans="1:4" ht="32.4">
       <c r="A46" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>59</v>
+        <v>97</v>
+      </c>
+      <c r="B46" s="31" t="s">
+        <v>98</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:4" ht="32.4">
+    <row r="47" spans="1:4">
       <c r="A47" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>53</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="1:4">
-      <c r="A48" s="9" t="s">
-        <v>96</v>
+    <row r="48" spans="1:4" ht="16.2" customHeight="1">
+      <c r="A48" s="19" t="s">
+        <v>55</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
     </row>
-    <row r="49" spans="1:4" ht="32.4">
+    <row r="49" spans="1:3" ht="48.6">
       <c r="A49" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B49" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-    </row>
-    <row r="50" spans="1:4">
-      <c r="A50" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-    </row>
-    <row r="51" spans="1:4" ht="16.2" customHeight="1">
-      <c r="A51" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-    </row>
-    <row r="52" spans="1:4" ht="48.6">
-      <c r="A52" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B52" s="20" t="s">
+      <c r="B49" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="C52" s="11" t="s">
+      <c r="C49" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="32.4">
-      <c r="A53" s="5" t="s">
+    <row r="50" spans="1:3" ht="32.4">
+      <c r="A50" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B53" s="12" t="s">
+      <c r="B50" s="12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
-      <c r="A54" s="50" t="s">
+    <row r="51" spans="1:3">
+      <c r="A51" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B51" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
-      <c r="A55" s="51"/>
+    <row r="52" spans="1:3">
+      <c r="A52" s="46"/>
+      <c r="B52" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54" s="15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="13" t="s">
+        <v>20</v>
+      </c>
       <c r="B55" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
       <c r="A56" s="13" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4">
-      <c r="A57" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B57" s="15" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
       <c r="A58" s="13" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4">
-      <c r="A59" s="13" t="s">
-        <v>22</v>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="51" t="s">
+        <v>28</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4">
-      <c r="A60" s="13" t="s">
-        <v>24</v>
-      </c>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
+      <c r="A60" s="45"/>
       <c r="B60" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4">
-      <c r="A61" s="13" t="s">
-        <v>26</v>
-      </c>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="46"/>
       <c r="B61" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4">
-      <c r="A62" s="50" t="s">
-        <v>28</v>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3">
+      <c r="A62" s="51" t="s">
+        <v>32</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4">
-      <c r="A63" s="52"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3">
+      <c r="A63" s="45"/>
       <c r="B63" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4">
-      <c r="A64" s="51"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3">
+      <c r="A64" s="45"/>
       <c r="B64" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2">
-      <c r="A65" s="50" t="s">
-        <v>32</v>
-      </c>
-      <c r="B65" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="46"/>
+      <c r="B65" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="51" t="s">
+        <v>37</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
-      <c r="A66" s="52"/>
-      <c r="B66" s="1" t="s">
+    <row r="67" spans="1:4">
+      <c r="A67" s="45"/>
+      <c r="B67" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
-      <c r="A67" s="52"/>
-      <c r="B67" s="1" t="s">
+    <row r="68" spans="1:4">
+      <c r="A68" s="45"/>
+      <c r="B68" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
-      <c r="A68" s="51"/>
-      <c r="B68" s="15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2">
-      <c r="A69" s="50" t="s">
-        <v>37</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2">
-      <c r="A70" s="52"/>
-      <c r="B70" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2">
-      <c r="A71" s="52"/>
+    <row r="69" spans="1:4">
+      <c r="A69" s="45"/>
+      <c r="B69" s="15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="46"/>
+      <c r="B70" s="15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="44" t="s">
+        <v>40</v>
+      </c>
       <c r="B71" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2">
-      <c r="A72" s="52"/>
-      <c r="B72" s="15" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2">
-      <c r="A73" s="51"/>
-      <c r="B73" s="15" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2">
-      <c r="A74" s="56" t="s">
-        <v>40</v>
-      </c>
-      <c r="B74" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="75" spans="1:2">
-      <c r="A75" s="52"/>
-      <c r="B75" s="1" t="s">
+    <row r="72" spans="1:4">
+      <c r="A72" s="45"/>
+      <c r="B72" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
-      <c r="A76" s="51"/>
-      <c r="B76" s="1" t="s">
+    <row r="73" spans="1:4">
+      <c r="A73" s="46"/>
+      <c r="B73" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="77" spans="1:2" ht="32.4">
-      <c r="A77" s="56" t="s">
+    <row r="74" spans="1:4" ht="32.4">
+      <c r="A74" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="B77" s="15" t="s">
+      <c r="B74" s="15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="78" spans="1:2" ht="32.4">
-      <c r="A78" s="52"/>
-      <c r="B78" s="15" t="s">
+    <row r="75" spans="1:4" ht="32.4">
+      <c r="A75" s="45"/>
+      <c r="B75" s="15" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="79" spans="1:2" ht="48.6">
-      <c r="A79" s="52"/>
-      <c r="B79" s="6" t="s">
+    <row r="76" spans="1:4" ht="48.6">
+      <c r="A76" s="45"/>
+      <c r="B76" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="80" spans="1:2">
-      <c r="A80" s="51"/>
-      <c r="B80" s="6" t="s">
+    <row r="77" spans="1:4">
+      <c r="A77" s="46"/>
+      <c r="B77" s="6" t="s">
         <v>48</v>
       </c>
     </row>
+    <row r="78" spans="1:4">
+      <c r="A78" s="62" t="s">
+        <v>61</v>
+      </c>
+      <c r="B78" s="53"/>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="A79" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B79" s="2"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2"/>
+    </row>
+    <row r="80" spans="1:4">
+      <c r="A80" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B80" s="16"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2"/>
+    </row>
     <row r="81" spans="1:4">
-      <c r="A81" s="43" t="s">
-        <v>61</v>
-      </c>
-      <c r="B81" s="44"/>
+      <c r="A81" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="B81" s="16"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
     </row>
     <row r="82" spans="1:4">
-      <c r="A82" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B82" s="2"/>
+      <c r="A82" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="B82" s="16"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="16" t="s">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="B83" s="16"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
     </row>
     <row r="84" spans="1:4">
-      <c r="A84" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="B84" s="16"/>
+      <c r="A84" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
     </row>
     <row r="85" spans="1:4">
-      <c r="A85" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="B85" s="16"/>
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
     </row>
-    <row r="86" spans="1:4">
-      <c r="A86" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="B86" s="16"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-    </row>
-    <row r="87" spans="1:4">
-      <c r="A87" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-    </row>
-    <row r="88" spans="1:4">
-      <c r="A88" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-    </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A66:A70"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="A34:A35"/>
     <mergeCell ref="A19:A20"/>
     <mergeCell ref="A27:A33"/>
-    <mergeCell ref="A74:A76"/>
-    <mergeCell ref="A77:A80"/>
+    <mergeCell ref="A71:A73"/>
+    <mergeCell ref="A74:A77"/>
     <mergeCell ref="D1:H2"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="E15:E16"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="A65:A68"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A62:A65"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:A13"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B13:B16"/>
-    <mergeCell ref="A81:B81"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A43"/>
-    <mergeCell ref="A54:A55"/>
-    <mergeCell ref="A69:A73"/>
   </mergeCells>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>

<commit_message>
Base.xlsx に refersTo と retrieve を定義し、Ontology.xlsx の agent などを retrieve の下位属性にする
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ontology/Base.xlsx
+++ b/ontology/Base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\home\doc\PLR\dist\schemata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA3F03A-7DCA-4B8A-9F7C-161952D9B303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F20951B-48ED-4656-B9BE-A610560CCDC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="15576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -465,11 +465,11 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>refersTo</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>retrieve retrieve</t>
+    <t>refersTo ja:参照;refers to</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>retrieve ja:検索;retrieve</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -1041,6 +1041,9 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1048,9 +1051,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1718,7 +1718,7 @@
       <c r="D34" s="2"/>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="67"/>
+      <c r="A35" s="64"/>
       <c r="B35" s="69"/>
       <c r="C35" s="34" t="s">
         <v>105</v>
@@ -1726,7 +1726,7 @@
       <c r="D35" s="2"/>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" s="64" t="s">
+      <c r="A36" s="65" t="s">
         <v>77</v>
       </c>
       <c r="B36" s="26" t="s">
@@ -1736,7 +1736,7 @@
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="65"/>
+      <c r="A37" s="66"/>
       <c r="B37" s="25" t="s">
         <v>78</v>
       </c>
@@ -1746,7 +1746,7 @@
       <c r="D37" s="2"/>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="65"/>
+      <c r="A38" s="66"/>
       <c r="B38" s="25" t="s">
         <v>84</v>
       </c>
@@ -1756,7 +1756,7 @@
       <c r="D38" s="2"/>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="65"/>
+      <c r="A39" s="66"/>
       <c r="B39" s="25" t="s">
         <v>80</v>
       </c>
@@ -1766,7 +1766,7 @@
       <c r="D39" s="2"/>
     </row>
     <row r="40" spans="1:4">
-      <c r="A40" s="66"/>
+      <c r="A40" s="67"/>
       <c r="B40" s="25" t="s">
         <v>82</v>
       </c>

</xml_diff>

<commit_message>
Base.xlsx・Ontology.xlsx：reuse（新規作成不可）を retrieve にまとめる——onto・ontoR00・ontoER・ontoEC と compensatesWith を retrieve の下位にする。reusable は当面残す（追記R788）
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ontology/Base.xlsx
+++ b/ontology/Base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\home\doc\PLR\dist\schemata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62390A3-4B84-4631-A435-4DA9F22B437B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E6E5E8D-91DC-4BDC-AFC6-6AB54E5CEAB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="15576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="125">
   <si>
     <t>dateTime</t>
   </si>
@@ -363,14 +363,6 @@
   </si>
   <si>
     <t>reusable ja:再利用可;reusable</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>reuse ja:再利用;reuse||ja:新規作成不可;no creation</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
-    <t>\(同じ値域の)異なる属性の値を再利用</t>
     <phoneticPr fontId="2"/>
   </si>
   <si>
@@ -999,23 +991,71 @@
     <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1028,16 +1068,10 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1061,48 +1095,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1425,7 +1417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30509B9C-F985-4EE4-8893-AAEEF9CB070C}">
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="16.2"/>
   <cols>
     <col min="1" max="1" width="38.88671875" style="17" customWidth="1"/>
@@ -1437,21 +1429,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.6" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="64" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="50"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="44" t="s">
-        <v>120</v>
-      </c>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
+      <c r="D1" s="60" t="s">
+        <v>118</v>
+      </c>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
     </row>
     <row r="2" spans="1:8" ht="39" customHeight="1">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="65" t="s">
         <v>86</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1460,14 +1452,14 @@
       <c r="C2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="52"/>
+      <c r="A3" s="66"/>
       <c r="B3" s="5" t="s">
         <v>90</v>
       </c>
@@ -1477,7 +1469,7 @@
       <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="52"/>
+      <c r="A4" s="66"/>
       <c r="B4" s="21" t="s">
         <v>1</v>
       </c>
@@ -1487,7 +1479,7 @@
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="52"/>
+      <c r="A5" s="66"/>
       <c r="B5" s="23" t="s">
         <v>73</v>
       </c>
@@ -1497,8 +1489,8 @@
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="52"/>
-      <c r="B6" s="53" t="s">
+      <c r="A6" s="66"/>
+      <c r="B6" s="67" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1507,23 +1499,23 @@
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="52"/>
-      <c r="B7" s="54"/>
+      <c r="A7" s="66"/>
+      <c r="B7" s="68"/>
       <c r="C7" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="52"/>
-      <c r="B8" s="55"/>
+      <c r="A8" s="66"/>
+      <c r="B8" s="69"/>
       <c r="C8" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="52"/>
+      <c r="A9" s="66"/>
       <c r="B9" s="7" t="s">
         <v>7</v>
       </c>
@@ -1533,8 +1525,8 @@
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="52"/>
-      <c r="B10" s="56" t="s">
+      <c r="A10" s="66"/>
+      <c r="B10" s="70" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -1543,15 +1535,15 @@
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="52"/>
-      <c r="B11" s="57"/>
+      <c r="A11" s="66"/>
+      <c r="B11" s="71"/>
       <c r="C11" s="7" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="52"/>
+      <c r="A12" s="66"/>
       <c r="B12" s="18" t="s">
         <v>57</v>
       </c>
@@ -1561,48 +1553,48 @@
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:8" ht="16.2" customHeight="1">
-      <c r="A13" s="52"/>
-      <c r="B13" s="58" t="s">
-        <v>102</v>
-      </c>
-      <c r="C13" s="69" t="s">
-        <v>106</v>
-      </c>
-      <c r="D13" s="72" t="s">
-        <v>124</v>
+      <c r="A13" s="66"/>
+      <c r="B13" s="72" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="43" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="16.2" customHeight="1">
       <c r="A14" s="33"/>
-      <c r="B14" s="58"/>
-      <c r="C14" s="70" t="s">
-        <v>101</v>
-      </c>
-      <c r="D14" s="72" t="s">
-        <v>124</v>
+      <c r="B14" s="72"/>
+      <c r="C14" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="D14" s="43" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="33"/>
-      <c r="B15" s="58"/>
-      <c r="C15" s="45" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" s="71" t="s">
+      <c r="B15" s="72"/>
+      <c r="C15" s="61" t="s">
+        <v>113</v>
+      </c>
+      <c r="D15" s="42" t="s">
+        <v>114</v>
+      </c>
+      <c r="E15" s="63" t="s">
         <v>116</v>
-      </c>
-      <c r="E15" s="47" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="33"/>
-      <c r="B16" s="58"/>
-      <c r="C16" s="46"/>
+      <c r="B16" s="72"/>
+      <c r="C16" s="62"/>
       <c r="D16" s="37" t="s">
-        <v>117</v>
-      </c>
-      <c r="E16" s="47"/>
+        <v>115</v>
+      </c>
+      <c r="E16" s="63"/>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="22" t="s">
@@ -1619,26 +1611,26 @@
         <v>95</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="56" t="s">
         <v>62</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="64.8">
-      <c r="A20" s="38"/>
+      <c r="A20" s="56"/>
       <c r="B20" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>64</v>
@@ -1646,7 +1638,7 @@
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B21" s="29" t="s">
         <v>94</v>
@@ -1699,444 +1691,442 @@
       <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4" ht="17.399999999999999">
-      <c r="A27" s="39" t="s">
-        <v>107</v>
+      <c r="A27" s="57" t="s">
+        <v>105</v>
       </c>
       <c r="B27" s="36" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C27" s="32"/>
       <c r="D27" s="32"/>
     </row>
     <row r="28" spans="1:4" ht="17.399999999999999">
-      <c r="A28" s="40"/>
+      <c r="A28" s="58"/>
       <c r="B28" s="36" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C28" s="32"/>
       <c r="D28" s="32"/>
     </row>
     <row r="29" spans="1:4" ht="17.399999999999999">
-      <c r="A29" s="40"/>
+      <c r="A29" s="58"/>
       <c r="B29" s="36" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C29" s="32"/>
       <c r="D29" s="32"/>
     </row>
     <row r="30" spans="1:4" ht="17.399999999999999">
-      <c r="A30" s="40"/>
+      <c r="A30" s="58"/>
       <c r="B30" s="36" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C30" s="32"/>
       <c r="D30" s="32"/>
     </row>
     <row r="31" spans="1:4" ht="17.399999999999999">
-      <c r="A31" s="40"/>
+      <c r="A31" s="58"/>
       <c r="B31" s="36" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C31" s="32"/>
       <c r="D31" s="32"/>
     </row>
     <row r="32" spans="1:4" ht="17.399999999999999">
-      <c r="A32" s="40"/>
+      <c r="A32" s="58"/>
       <c r="B32" s="36" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C32" s="32"/>
       <c r="D32" s="32"/>
     </row>
     <row r="33" spans="1:4" ht="17.399999999999999">
-      <c r="A33" s="40"/>
+      <c r="A33" s="58"/>
       <c r="B33" s="36" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C33" s="32"/>
       <c r="D33" s="32"/>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="60" t="s">
-        <v>122</v>
-      </c>
-      <c r="B34" s="65" t="s">
-        <v>123</v>
+      <c r="A34" s="54" t="s">
+        <v>120</v>
+      </c>
+      <c r="B34" s="52" t="s">
+        <v>121</v>
       </c>
       <c r="C34" s="34" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D34" s="2"/>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="61"/>
-      <c r="B35" s="66"/>
+      <c r="A35" s="55"/>
+      <c r="B35" s="53"/>
       <c r="C35" s="34" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D35" s="2"/>
     </row>
     <row r="36" spans="1:4">
-      <c r="A36" s="67" t="s">
-        <v>125</v>
+      <c r="A36" s="9" t="s">
+        <v>96</v>
       </c>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
     </row>
     <row r="37" spans="1:4">
-      <c r="A37" s="68" t="s">
-        <v>126</v>
+      <c r="A37" s="38" t="s">
+        <v>123</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="62" t="s">
-        <v>77</v>
-      </c>
-      <c r="B38" s="26" t="s">
-        <v>64</v>
-      </c>
+      <c r="A38" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
     </row>
     <row r="39" spans="1:4">
-      <c r="A39" s="63"/>
-      <c r="B39" s="25" t="s">
+      <c r="A39" s="46" t="s">
+        <v>77</v>
+      </c>
+      <c r="B39" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="47"/>
+      <c r="B40" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C40" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D39" s="2"/>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="63"/>
-      <c r="B40" s="25" t="s">
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="47"/>
+      <c r="B41" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C41" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="D40" s="2"/>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="63"/>
-      <c r="B41" s="25" t="s">
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="47"/>
+      <c r="B42" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C42" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="D41" s="2"/>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="64"/>
-      <c r="B42" s="25" t="s">
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="48"/>
+      <c r="B43" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C43" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="D42" s="2"/>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="24" t="s">
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="24" t="s">
         <v>63</v>
-      </c>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="B44" s="25" t="s">
-        <v>76</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
     </row>
     <row r="45" spans="1:4">
-      <c r="A45" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B45" s="10" t="s">
-        <v>59</v>
+      <c r="A45" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="B45" s="25" t="s">
+        <v>76</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:4" ht="32.4">
+    <row r="46" spans="1:4">
       <c r="A46" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>53</v>
+        <v>58</v>
+      </c>
+      <c r="B46" s="10" t="s">
+        <v>59</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:4">
+    <row r="47" spans="1:4" ht="32.4">
       <c r="A47" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B47" s="2"/>
+        <v>93</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>53</v>
+      </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
     </row>
-    <row r="48" spans="1:4" ht="32.4">
+    <row r="48" spans="1:4">
       <c r="A48" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B48" s="31" t="s">
-        <v>98</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
     </row>
-    <row r="49" spans="1:4">
-      <c r="A49" s="9" t="s">
-        <v>54</v>
+    <row r="49" spans="1:4" ht="16.2" customHeight="1">
+      <c r="A49" s="19" t="s">
+        <v>55</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
     </row>
-    <row r="50" spans="1:4" ht="16.2" customHeight="1">
-      <c r="A50" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-    </row>
-    <row r="51" spans="1:4" ht="48.6">
-      <c r="A51" s="9" t="s">
+    <row r="50" spans="1:4" ht="48.6">
+      <c r="A50" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B51" s="20" t="s">
+      <c r="B50" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C50" s="11" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="32.4">
-      <c r="A52" s="5" t="s">
+    <row r="51" spans="1:4" ht="32.4">
+      <c r="A51" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B52" s="12" t="s">
+      <c r="B51" s="12" t="s">
         <v>12</v>
       </c>
     </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
     <row r="53" spans="1:4">
-      <c r="A53" s="48" t="s">
-        <v>13</v>
-      </c>
+      <c r="A53" s="50"/>
       <c r="B53" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" s="43"/>
+      <c r="A54" s="13" t="s">
+        <v>16</v>
+      </c>
       <c r="B54" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:4">
-      <c r="A55" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>17</v>
+      <c r="A55" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B55" s="15" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="56" spans="1:4">
-      <c r="A56" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B56" s="15" t="s">
-        <v>19</v>
+      <c r="A56" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="13" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:4">
-      <c r="A60" s="13" t="s">
-        <v>26</v>
+      <c r="A60" s="49" t="s">
+        <v>28</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="61" spans="1:4">
-      <c r="A61" s="48" t="s">
-        <v>28</v>
-      </c>
+      <c r="A61" s="51"/>
       <c r="B61" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="62" spans="1:4">
-      <c r="A62" s="42"/>
+      <c r="A62" s="50"/>
       <c r="B62" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="63" spans="1:4">
-      <c r="A63" s="43"/>
+      <c r="A63" s="49" t="s">
+        <v>32</v>
+      </c>
       <c r="B63" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="64" spans="1:4">
-      <c r="A64" s="48" t="s">
-        <v>32</v>
-      </c>
+      <c r="A64" s="51"/>
       <c r="B64" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4">
+      <c r="A65" s="51"/>
+      <c r="B65" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4">
+      <c r="A66" s="50"/>
+      <c r="B66" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4">
+      <c r="A67" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="65" spans="1:4">
-      <c r="A65" s="42"/>
-      <c r="B65" s="1" t="s">
+    <row r="68" spans="1:4">
+      <c r="A68" s="51"/>
+      <c r="B68" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="66" spans="1:4">
-      <c r="A66" s="42"/>
-      <c r="B66" s="1" t="s">
+    <row r="69" spans="1:4">
+      <c r="A69" s="51"/>
+      <c r="B69" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="67" spans="1:4">
-      <c r="A67" s="43"/>
-      <c r="B67" s="15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4">
-      <c r="A68" s="48" t="s">
-        <v>37</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4">
-      <c r="A69" s="42"/>
-      <c r="B69" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
     <row r="70" spans="1:4">
-      <c r="A70" s="42"/>
-      <c r="B70" s="1" t="s">
-        <v>35</v>
+      <c r="A70" s="51"/>
+      <c r="B70" s="15" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="71" spans="1:4">
-      <c r="A71" s="42"/>
+      <c r="A71" s="50"/>
       <c r="B71" s="15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="72" spans="1:4">
-      <c r="A72" s="43"/>
-      <c r="B72" s="15" t="s">
-        <v>39</v>
+      <c r="A72" s="59" t="s">
+        <v>40</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="73" spans="1:4">
-      <c r="A73" s="41" t="s">
-        <v>40</v>
-      </c>
+      <c r="A73" s="51"/>
       <c r="B73" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="74" spans="1:4">
-      <c r="A74" s="42"/>
+      <c r="A74" s="50"/>
       <c r="B74" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4">
-      <c r="A75" s="43"/>
-      <c r="B75" s="1" t="s">
         <v>43</v>
       </c>
     </row>
+    <row r="75" spans="1:4" ht="32.4">
+      <c r="A75" s="59" t="s">
+        <v>44</v>
+      </c>
+      <c r="B75" s="15" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="76" spans="1:4" ht="32.4">
-      <c r="A76" s="41" t="s">
-        <v>44</v>
-      </c>
+      <c r="A76" s="51"/>
       <c r="B76" s="15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="32.4">
-      <c r="A77" s="42"/>
-      <c r="B77" s="15" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="48.6">
-      <c r="A78" s="42"/>
+    <row r="77" spans="1:4" ht="48.6">
+      <c r="A77" s="51"/>
+      <c r="B77" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="A78" s="50"/>
       <c r="B78" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="79" spans="1:4">
-      <c r="A79" s="43"/>
-      <c r="B79" s="6" t="s">
-        <v>48</v>
-      </c>
+      <c r="A79" s="44" t="s">
+        <v>61</v>
+      </c>
+      <c r="B79" s="45"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2"/>
     </row>
     <row r="80" spans="1:4">
-      <c r="A80" s="59" t="s">
-        <v>61</v>
-      </c>
-      <c r="B80" s="50"/>
+      <c r="A80" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
     </row>
     <row r="81" spans="1:4">
-      <c r="A81" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B81" s="2"/>
+      <c r="A81" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B81" s="16"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2"/>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B82" s="16"/>
       <c r="C82" s="2"/>
@@ -2144,7 +2134,7 @@
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B83" s="16"/>
       <c r="C83" s="2"/>
@@ -2152,58 +2142,50 @@
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="16" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="B84" s="16"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2"/>
     </row>
     <row r="85" spans="1:4">
-      <c r="A85" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="B85" s="16"/>
+      <c r="A85" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2"/>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="2" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
     </row>
-    <row r="87" spans="1:4">
-      <c r="A87" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-    </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A80:B80"/>
-    <mergeCell ref="A38:A42"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A68:A72"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="A34:A35"/>
     <mergeCell ref="A19:A20"/>
     <mergeCell ref="A27:A33"/>
-    <mergeCell ref="A73:A75"/>
-    <mergeCell ref="A76:A79"/>
+    <mergeCell ref="A72:A74"/>
+    <mergeCell ref="A75:A78"/>
     <mergeCell ref="D1:H2"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="E15:E16"/>
-    <mergeCell ref="A61:A63"/>
-    <mergeCell ref="A64:A67"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="A63:A66"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:A13"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="B13:B16"/>
+    <mergeCell ref="A79:B79"/>
+    <mergeCell ref="A39:A43"/>
+    <mergeCell ref="A52:A53"/>
+    <mergeCell ref="A67:A71"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="A34:A35"/>
   </mergeCells>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>